<commit_message>
Fix SharePoint list import: unambiguous example values
SharePoint's 'From Excel' import rejected the Companies example row when
a value didn't match its guessed column type. Example values are now
plainly text (no URL-like or number-like strings, no empty cells), and
the Read me lists the exact column type for every column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018jLnLSVt3GVsxGmUeG6jXM
</commit_message>
<xml_diff>
--- a/powerapps/sharepoint-lists-setup.xlsx
+++ b/powerapps/sharepoint-lists-setup.xlsx
@@ -666,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -699,64 +699,85 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>3. Check the column types SharePoint suggests: dates must be 'Date and time', numbers 'Number',</t>
+          <t>3. Before clicking Create, check each column's type in the panel on the right:</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   long text (Notes, Summary, Statement, Includes) may be 'Multiple lines of text', all else 'Single line of text'.</t>
+          <t xml:space="preserve">   - Number: F1, F2, F3, F5, AmountDKK, ProposedDKK, AgreedDKK, PriceDKK, CapacityPerSemester, Attendance</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4. Name the list exactly like the table (Companies, CommercialEvidence, Contacts, Opportunities,</t>
+          <t xml:space="preserve">   - Date and time: columns ending in On, Date, Due, Until, Start or End (e.g. FitReviewedOn, NextActionDue, TermStart)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Interactions, Evidence, TeamMembers, Packages, Themes, Events, Settings). Repeat for every table.</t>
+          <t xml:space="preserve">   - Everything else: Single line of text (change 'Hyperlink', 'Person', 'Choice' or 'Yes/No' to Single line of text)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5. Delete the example rows (marked '(example)') in each list. Keep all Settings rows and edit their values.</t>
+          <t xml:space="preserve">   If SharePoint says a row was omitted, that's only the example row: check the column types and carry on.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>4. Name the list exactly like the table (Companies, CommercialEvidence, Contacts, Opportunities,</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Column names have no spaces on purpose: the Power Apps formulas use these exact names.</t>
+          <t xml:space="preserve">   Interactions, Evidence, TeamMembers, Packages, Themes, Events, Settings). Repeat for every table.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Allowed values (Stage, Outcome, EvidenceType, ...) are enforced by the app's dropdowns,</t>
+          <t>5. Delete the example rows (marked '(example)') in each list. Keep all Settings rows and edit their values.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>so SharePoint columns stay plain text. See docs/powerapps-data-model.md in the repository.</t>
-        </is>
-      </c>
+      <c r="A13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Column names have no spaces on purpose: the Power Apps formulas use these exact names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Allowed values (Stage, Outcome, EvidenceType, ...) are enforced by the app's dropdowns,</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>so SharePoint columns stay plain text. See docs/powerapps-data-model.md in the repository.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>All example data is fictional.</t>
         </is>
@@ -900,7 +921,11 @@
           <t>BSc IB 25%, MSc FIN 15%, other 60%</t>
         </is>
       </c>
-      <c r="F2" s="4" t="n"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="G2" s="5" t="n">
         <v>46307</v>
       </c>
@@ -1261,12 +1286,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>nordlys.example</t>
+          <t>Nordlys website (example)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>12345678</t>
+          <t>CVR (example)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -1276,7 +1301,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>250-999</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1292,7 +1317,11 @@
           <t>Relevant to supply-chain students</t>
         </is>
       </c>
-      <c r="I2" s="4" t="n"/>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="J2" s="4" t="n">
         <v>1</v>
       </c>
@@ -1301,7 +1330,11 @@
           <t>Supply-chain topic, no named speaker yet</t>
         </is>
       </c>
-      <c r="L2" s="4" t="n"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="M2" s="4" t="n">
         <v>2</v>
       </c>
@@ -1312,7 +1345,7 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>https://example.org/jobs</t>
+          <t>Company jobs page (example)</t>
         </is>
       </c>
       <c r="P2" s="4" t="n">
@@ -1325,7 +1358,7 @@
       </c>
       <c r="R2" s="4" t="inlineStr">
         <is>
-          <t>https://example.org/graduates</t>
+          <t>Company careers page (example)</t>
         </is>
       </c>
       <c r="S2" s="5" t="n">
@@ -1336,23 +1369,39 @@
           <t>CBS alumnus in their talent team, via A.K. (agreed)</t>
         </is>
       </c>
-      <c r="U2" s="4" t="n"/>
+      <c r="U2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="W2" s="4" t="n"/>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="X2" s="5" t="n">
         <v>46307</v>
       </c>
-      <c r="Y2" s="4" t="n"/>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AA2" s="4" t="n"/>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1439,7 +1488,11 @@
           <t>Checked partner pages of 12 CBS student organisations</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n"/>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="E2" s="4" t="n">
         <v>0</v>
       </c>
@@ -1581,8 +1634,16 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Company team page</t>
@@ -1797,7 +1858,11 @@
           <t>Non-cash</t>
         </is>
       </c>
-      <c r="H2" s="4" t="n"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="I2" s="4" t="n">
         <v>0</v>
       </c>
@@ -1831,9 +1896,21 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="U2" s="5" t="n">
         <v>46307</v>
       </c>
@@ -2051,10 +2128,14 @@
           <t>Verified fact</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n"/>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>https://example.org/jobs</t>
+          <t>Company jobs page (example)</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -2139,7 +2220,11 @@
           <t>Partnerships Manager</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n"/>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>(example)</t>
+        </is>
+      </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Yes</t>

</xml_diff>